<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.32-1-lts #1 SMP PREEMPT_DYNAMIC Sat, 25 May 2024 20:20:51 +0000 x86_64 GNU/Linux  13:21:03 up  2:27,  1 user,  load average: 1.97, 1.06, 0.98
</commit_message>
<xml_diff>
--- a/npc/tools/exu_gen/exu_table.xlsx
+++ b/npc/tools/exu_gen/exu_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="89">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="104">
   <si>
     <t>commont</t>
   </si>
@@ -61,6 +61,18 @@
     <t>sranum</t>
   </si>
   <si>
+    <t>csr_raddr</t>
+  </si>
+  <si>
+    <t>csr_we</t>
+  </si>
+  <si>
+    <t>csr_waddr</t>
+  </si>
+  <si>
+    <t>csr_wdata</t>
+  </si>
+  <si>
     <t>`Inst_addi</t>
   </si>
   <si>
@@ -269,6 +281,39 @@
   </si>
   <si>
     <t>`Inst_sw</t>
+  </si>
+  <si>
+    <t>`Inst_csrrw</t>
+  </si>
+  <si>
+    <t>csr_rdata</t>
+  </si>
+  <si>
+    <t>imm[11:0]</t>
+  </si>
+  <si>
+    <t>src1</t>
+  </si>
+  <si>
+    <t>`Inst_csrrs</t>
+  </si>
+  <si>
+    <t>src1|csr_rdata</t>
+  </si>
+  <si>
+    <t>//此处只设置pc偏移,余下部分在csr模块中</t>
+  </si>
+  <si>
+    <t>`Inst_ecall</t>
+  </si>
+  <si>
+    <t>csr_rdata-exu_pc</t>
+  </si>
+  <si>
+    <t>`MTVEC_NO</t>
+  </si>
+  <si>
+    <t>`Inst_mret</t>
   </si>
   <si>
     <t>default</t>
@@ -288,15 +333,36 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="20">
+  <fonts count="21">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.8"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -317,85 +383,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -410,7 +399,55 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -425,15 +462,15 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FF0000FF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -445,6 +482,20 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="35">
     <fill>
@@ -467,37 +518,175 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -510,144 +699,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -658,6 +709,24 @@
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -685,6 +754,17 @@
       <diagonal/>
     </border>
     <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color rgb="FFB2B2B2"/>
       </left>
@@ -700,22 +780,17 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
       <top style="thin">
-        <color theme="4"/>
+        <color rgb="FF3F3F3F"/>
       </top>
-      <bottom style="double">
-        <color theme="4"/>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -734,181 +809,157 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="2" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="21" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="19" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -932,6 +983,9 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1252,10 +1306,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:T55"/>
+  <dimension ref="A1:S59"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="11.875" customWidth="1"/>
+    <col min="1" max="1" width="32.625" customWidth="1"/>
     <col min="2" max="2" width="17.7583333333333" customWidth="1"/>
     <col min="3" max="3" width="10.1416666666667" customWidth="1"/>
     <col min="4" max="4" width="13.1416666666667" customWidth="1"/>
@@ -1269,12 +1323,13 @@
     <col min="13" max="13" width="11.8083333333333" customWidth="1"/>
     <col min="14" max="14" width="10.6" customWidth="1"/>
     <col min="15" max="15" width="9.70833333333333" customWidth="1"/>
-    <col min="16" max="16" width="11.7083333333333" customWidth="1"/>
-    <col min="18" max="18" width="11.4083333333333" customWidth="1"/>
-    <col min="19" max="20" width="12.0583333333333" customWidth="1"/>
+    <col min="16" max="16" width="11.1666666666667" customWidth="1"/>
+    <col min="17" max="17" width="11.4083333333333" customWidth="1"/>
+    <col min="18" max="18" width="12.0583333333333" customWidth="1"/>
+    <col min="19" max="19" width="15.575" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" spans="1:15">
+    <row r="1" ht="15" customHeight="1" spans="1:19">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1320,19 +1375,31 @@
       <c r="O1" s="2" t="s">
         <v>14</v>
       </c>
+      <c r="P1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="2" spans="2:15">
       <c r="B2" s="2" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
@@ -1347,16 +1414,16 @@
     </row>
     <row r="3" spans="2:15">
       <c r="B3" s="2" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
@@ -1371,16 +1438,16 @@
     </row>
     <row r="4" spans="2:15">
       <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="E4" s="2" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
@@ -1395,16 +1462,16 @@
     </row>
     <row r="5" spans="2:15">
       <c r="B5" s="2" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1419,16 +1486,16 @@
     </row>
     <row r="6" spans="2:15">
       <c r="B6" s="2" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="F6" s="2"/>
       <c r="G6" s="2"/>
@@ -1444,22 +1511,22 @@
     <row r="7" s="1" customFormat="1" spans="1:15">
       <c r="A7"/>
       <c r="B7" s="3" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="H7" s="3"/>
       <c r="I7" s="3"/>
@@ -1473,22 +1540,22 @@
     <row r="8" s="1" customFormat="1" spans="1:15">
       <c r="A8"/>
       <c r="B8" s="3" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -1501,16 +1568,16 @@
     </row>
     <row r="9" spans="2:15">
       <c r="B9" s="2" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
       <c r="E9" s="2"/>
       <c r="F9" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
@@ -1523,16 +1590,16 @@
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="2" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
       <c r="E10" s="2"/>
       <c r="F10" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="H10" s="2"/>
       <c r="I10" s="2"/>
@@ -1545,16 +1612,16 @@
     </row>
     <row r="11" spans="2:15">
       <c r="B11" s="2" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
       <c r="E11" s="2"/>
       <c r="F11" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
@@ -1567,16 +1634,16 @@
     </row>
     <row r="12" spans="2:15">
       <c r="B12" s="2" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
@@ -1589,16 +1656,16 @@
     </row>
     <row r="13" spans="2:15">
       <c r="B13" s="2" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
       <c r="F13" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -1611,16 +1678,16 @@
     </row>
     <row r="14" spans="2:15">
       <c r="B14" s="2" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
       <c r="F14" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -1633,16 +1700,16 @@
     </row>
     <row r="15" spans="2:15">
       <c r="B15" s="2" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F15" s="2"/>
       <c r="G15" s="2"/>
@@ -1657,16 +1724,16 @@
     </row>
     <row r="16" spans="2:15">
       <c r="B16" s="2" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -1681,16 +1748,16 @@
     </row>
     <row r="17" spans="2:15">
       <c r="B17" s="2" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -1705,16 +1772,16 @@
     </row>
     <row r="18" spans="2:15">
       <c r="B18" s="2" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -1729,16 +1796,16 @@
     </row>
     <row r="19" spans="2:15">
       <c r="B19" s="2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -1753,16 +1820,16 @@
     </row>
     <row r="20" spans="2:15">
       <c r="B20" s="2" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -1777,16 +1844,16 @@
     </row>
     <row r="21" spans="2:15">
       <c r="B21" s="2" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -1801,16 +1868,16 @@
     </row>
     <row r="22" spans="2:15">
       <c r="B22" s="2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E22" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -1825,16 +1892,16 @@
     </row>
     <row r="23" spans="2:15">
       <c r="B23" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -1846,21 +1913,21 @@
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
       <c r="O23" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
     </row>
     <row r="24" spans="2:15">
       <c r="B24" s="2" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -1872,21 +1939,21 @@
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
       <c r="O24" s="2" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="25" spans="2:15">
       <c r="B25" s="2" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D25" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1901,16 +1968,16 @@
     </row>
     <row r="26" spans="2:15">
       <c r="B26" s="2" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -1925,16 +1992,16 @@
     </row>
     <row r="27" spans="2:15">
       <c r="B27" s="2" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D27" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E27" s="2" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="F27" s="2"/>
       <c r="G27" s="2"/>
@@ -1949,27 +2016,27 @@
     </row>
     <row r="28" spans="2:15">
       <c r="B28" s="2" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
       <c r="H28" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="J28" s="7" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
@@ -1979,27 +2046,27 @@
     </row>
     <row r="29" spans="2:15">
       <c r="B29" s="2" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
       <c r="H29" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
@@ -2009,27 +2076,27 @@
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="2" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D30" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
       <c r="H30" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
@@ -2039,27 +2106,27 @@
     </row>
     <row r="31" spans="2:15">
       <c r="B31" s="2" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D31" s="2" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
@@ -2069,7 +2136,7 @@
     </row>
     <row r="32" spans="2:15">
       <c r="B32" s="2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -2080,22 +2147,22 @@
       <c r="I32" s="2"/>
       <c r="J32" s="3"/>
       <c r="K32" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="L32" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="M32" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="N32" s="2" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="O32" s="2"/>
     </row>
     <row r="33" spans="2:15">
       <c r="B33" s="2" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -2106,22 +2173,22 @@
       <c r="I33" s="2"/>
       <c r="J33" s="2"/>
       <c r="K33" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="L33" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="O33" s="2"/>
     </row>
     <row r="34" spans="2:15">
       <c r="B34" s="2" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -2132,142 +2199,228 @@
       <c r="I34" s="2"/>
       <c r="J34" s="2"/>
       <c r="K34" s="2" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="O34" s="2"/>
     </row>
-    <row r="35" spans="2:15">
+    <row r="35" spans="2:19">
       <c r="B35" s="2" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>86</v>
+        <v>20</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>87</v>
+        <v>21</v>
       </c>
       <c r="E35" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F35" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="G35" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="H35" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="I35" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="J35" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="K35" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="L35" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="M35" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="N35" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="O35" s="2">
+        <v>90</v>
+      </c>
+      <c r="F35" s="2"/>
+      <c r="G35" s="2"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2"/>
+      <c r="J35" s="2"/>
+      <c r="K35" s="2"/>
+      <c r="L35" s="2"/>
+      <c r="M35" s="2"/>
+      <c r="N35" s="2"/>
+      <c r="O35" s="2"/>
+      <c r="P35" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>20</v>
+      </c>
+      <c r="R35" t="s">
+        <v>91</v>
+      </c>
+      <c r="S35" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="36" spans="2:19">
+      <c r="B36" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="F36" s="2"/>
+      <c r="G36" s="2"/>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2"/>
+      <c r="J36" s="2"/>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
+      <c r="O36" s="2"/>
+      <c r="P36" t="s">
+        <v>91</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>20</v>
+      </c>
+      <c r="R36" t="s">
+        <v>91</v>
+      </c>
+      <c r="S36" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="37" spans="1:16">
+      <c r="A37" t="s">
+        <v>95</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2"/>
+      <c r="J37" s="2"/>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
+      <c r="O37" s="2"/>
+      <c r="P37" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16">
+      <c r="A38" t="s">
+        <v>95</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2"/>
+      <c r="J38" s="2"/>
+      <c r="K38" s="2"/>
+      <c r="L38" s="2"/>
+      <c r="M38" s="2"/>
+      <c r="N38" s="2"/>
+      <c r="O38" s="2"/>
+      <c r="P38" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="39" spans="2:19">
+      <c r="B39" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="F39" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="I39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K39" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="L39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="M39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="O39" s="2">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" spans="1:20">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="N42" s="2"/>
-      <c r="P42" s="2"/>
-      <c r="Q42" s="2"/>
-      <c r="R42" s="2"/>
-      <c r="S42" s="2"/>
-      <c r="T42" s="2"/>
-    </row>
-    <row r="43" spans="1:20">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="N43" s="2"/>
-      <c r="O43" s="2"/>
-      <c r="P43" s="2"/>
-      <c r="Q43" s="2"/>
-      <c r="R43" s="2"/>
-      <c r="S43" s="2"/>
-      <c r="T43" s="2"/>
-    </row>
-    <row r="44" spans="1:20">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="N44" s="2"/>
-      <c r="O44" s="2"/>
-      <c r="P44" s="2"/>
-      <c r="Q44" s="2"/>
-      <c r="R44" s="2"/>
-      <c r="S44" s="2"/>
-      <c r="T44" s="2"/>
-    </row>
-    <row r="45" spans="1:20">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2"/>
-      <c r="P45" s="2"/>
-      <c r="Q45" s="2"/>
-      <c r="R45" s="2"/>
-      <c r="S45" s="2"/>
-      <c r="T45" s="2"/>
-    </row>
-    <row r="46" spans="1:20">
+      <c r="P39">
+        <v>0</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>101</v>
+      </c>
+      <c r="R39">
+        <v>0</v>
+      </c>
+      <c r="S39">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:19">
       <c r="A46" s="2"/>
       <c r="B46" s="2"/>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
       <c r="N46" s="2"/>
-      <c r="O46" s="2"/>
       <c r="P46" s="2"/>
       <c r="Q46" s="2"/>
       <c r="R46" s="2"/>
       <c r="S46" s="2"/>
-      <c r="T46" s="2"/>
-    </row>
-    <row r="47" spans="1:20">
+    </row>
+    <row r="47" spans="1:19">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
       <c r="P47" s="2"/>
       <c r="Q47" s="2"/>
       <c r="R47" s="2"/>
       <c r="S47" s="2"/>
-      <c r="T47" s="2"/>
-    </row>
-    <row r="48" spans="1:20">
+    </row>
+    <row r="48" spans="1:19">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
@@ -2278,9 +2431,8 @@
       <c r="Q48" s="2"/>
       <c r="R48" s="2"/>
       <c r="S48" s="2"/>
-      <c r="T48" s="2"/>
-    </row>
-    <row r="49" spans="1:20">
+    </row>
+    <row r="49" spans="1:19">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
@@ -2291,9 +2443,8 @@
       <c r="Q49" s="2"/>
       <c r="R49" s="2"/>
       <c r="S49" s="2"/>
-      <c r="T49" s="2"/>
-    </row>
-    <row r="50" spans="1:20">
+    </row>
+    <row r="50" spans="1:19">
       <c r="A50" s="2"/>
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
@@ -2304,9 +2455,8 @@
       <c r="Q50" s="2"/>
       <c r="R50" s="2"/>
       <c r="S50" s="2"/>
-      <c r="T50" s="2"/>
-    </row>
-    <row r="51" spans="1:20">
+    </row>
+    <row r="51" spans="1:19">
       <c r="A51" s="2"/>
       <c r="B51" s="2"/>
       <c r="C51" s="2"/>
@@ -2317,9 +2467,8 @@
       <c r="Q51" s="2"/>
       <c r="R51" s="2"/>
       <c r="S51" s="2"/>
-      <c r="T51" s="2"/>
-    </row>
-    <row r="52" spans="1:20">
+    </row>
+    <row r="52" spans="1:19">
       <c r="A52" s="2"/>
       <c r="B52" s="2"/>
       <c r="C52" s="2"/>
@@ -2330,9 +2479,8 @@
       <c r="Q52" s="2"/>
       <c r="R52" s="2"/>
       <c r="S52" s="2"/>
-      <c r="T52" s="2"/>
-    </row>
-    <row r="53" spans="1:20">
+    </row>
+    <row r="53" spans="1:19">
       <c r="A53" s="2"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -2343,9 +2491,8 @@
       <c r="Q53" s="2"/>
       <c r="R53" s="2"/>
       <c r="S53" s="2"/>
-      <c r="T53" s="2"/>
-    </row>
-    <row r="54" spans="1:20">
+    </row>
+    <row r="54" spans="1:19">
       <c r="A54" s="2"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -2356,9 +2503,8 @@
       <c r="Q54" s="2"/>
       <c r="R54" s="2"/>
       <c r="S54" s="2"/>
-      <c r="T54" s="2"/>
-    </row>
-    <row r="55" spans="1:20">
+    </row>
+    <row r="55" spans="1:19">
       <c r="A55" s="2"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -2369,7 +2515,54 @@
       <c r="Q55" s="2"/>
       <c r="R55" s="2"/>
       <c r="S55" s="2"/>
-      <c r="T55" s="2"/>
+    </row>
+    <row r="56" spans="1:19">
+      <c r="A56" s="2"/>
+      <c r="B56" s="2"/>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="N56" s="2"/>
+      <c r="O56" s="2"/>
+      <c r="P56" s="2"/>
+      <c r="Q56" s="2"/>
+      <c r="R56" s="2"/>
+      <c r="S56" s="2"/>
+    </row>
+    <row r="57" spans="1:19">
+      <c r="A57" s="2"/>
+      <c r="B57" s="2"/>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="N57" s="2"/>
+      <c r="O57" s="2"/>
+      <c r="P57" s="2"/>
+      <c r="Q57" s="2"/>
+      <c r="R57" s="2"/>
+      <c r="S57" s="2"/>
+    </row>
+    <row r="58" spans="1:19">
+      <c r="A58" s="2"/>
+      <c r="B58" s="2"/>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="N58" s="2"/>
+      <c r="O58" s="2"/>
+      <c r="P58" s="2"/>
+      <c r="Q58" s="2"/>
+      <c r="R58" s="2"/>
+      <c r="S58" s="2"/>
+    </row>
+    <row r="59" spans="1:19">
+      <c r="A59" s="2"/>
+      <c r="B59" s="2"/>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="N59" s="2"/>
+      <c r="O59" s="2"/>
+      <c r="P59" s="2"/>
+      <c r="Q59" s="2"/>
+      <c r="R59" s="2"/>
+      <c r="S59" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.32-1-lts #1 SMP PREEMPT_DYNAMIC Sat, 25 May 2024 20:20:51 +0000 x86_64 GNU/Linux  15:26:43 up  4:33,  1 user,  load average: 2.02, 2.03, 2.35
</commit_message>
<xml_diff>
--- a/npc/tools/exu_gen/exu_table.xlsx
+++ b/npc/tools/exu_gen/exu_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="106">
   <si>
     <t>commont</t>
   </si>
@@ -167,6 +167,12 @@
   </si>
   <si>
     <t>src1 ^ src2</t>
+  </si>
+  <si>
+    <t>`Inst_slt</t>
+  </si>
+  <si>
+    <t>$signed(src1)&lt;$signed(src2) ? 1 : 0</t>
   </si>
   <si>
     <t>`Inst_sltu</t>
@@ -1306,7 +1312,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S59"/>
+  <dimension ref="A1:S60"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="32.625" customWidth="1"/>
@@ -1900,7 +1906,7 @@
       <c r="D23" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E23" s="4" t="s">
+      <c r="E23" s="2" t="s">
         <v>64</v>
       </c>
       <c r="F23" s="2"/>
@@ -1912,13 +1918,11 @@
       <c r="L23" s="2"/>
       <c r="M23" s="2"/>
       <c r="N23" s="2"/>
-      <c r="O23" s="2" t="s">
-        <v>65</v>
-      </c>
+      <c r="O23" s="2"/>
     </row>
     <row r="24" spans="2:15">
       <c r="B24" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C24" s="2" t="s">
         <v>20</v>
@@ -1927,7 +1931,7 @@
         <v>21</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F24" s="2"/>
       <c r="G24" s="2"/>
@@ -1953,7 +1957,7 @@
         <v>21</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1964,7 +1968,9 @@
       <c r="L25" s="2"/>
       <c r="M25" s="2"/>
       <c r="N25" s="2"/>
-      <c r="O25" s="2"/>
+      <c r="O25" s="2" t="s">
+        <v>69</v>
+      </c>
     </row>
     <row r="26" spans="2:15">
       <c r="B26" s="2" t="s">
@@ -1976,7 +1982,7 @@
       <c r="D26" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="4" t="s">
         <v>71</v>
       </c>
       <c r="F26" s="2"/>
@@ -2029,15 +2035,9 @@
       </c>
       <c r="F28" s="2"/>
       <c r="G28" s="2"/>
-      <c r="H28" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J28" s="7" t="s">
-        <v>76</v>
-      </c>
+      <c r="H28" s="2"/>
+      <c r="I28" s="2"/>
+      <c r="J28" s="2"/>
       <c r="K28" s="2"/>
       <c r="L28" s="2"/>
       <c r="M28" s="2"/>
@@ -2046,7 +2046,7 @@
     </row>
     <row r="29" spans="2:15">
       <c r="B29" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C29" s="2" t="s">
         <v>20</v>
@@ -2055,7 +2055,7 @@
         <v>21</v>
       </c>
       <c r="E29" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
@@ -2066,7 +2066,7 @@
         <v>22</v>
       </c>
       <c r="J29" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
@@ -2076,7 +2076,7 @@
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>20</v>
@@ -2084,8 +2084,8 @@
       <c r="D30" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E30" s="5" t="s">
-        <v>81</v>
+      <c r="E30" s="2" t="s">
+        <v>80</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -2096,7 +2096,7 @@
         <v>22</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
@@ -2114,7 +2114,7 @@
       <c r="D31" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="6" t="s">
+      <c r="E31" s="5" t="s">
         <v>83</v>
       </c>
       <c r="F31" s="2"/>
@@ -2126,7 +2126,7 @@
         <v>22</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
@@ -2136,28 +2136,32 @@
     </row>
     <row r="32" spans="2:15">
       <c r="B32" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D32" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E32" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
-      <c r="H32" s="2"/>
-      <c r="I32" s="2"/>
-      <c r="J32" s="3"/>
-      <c r="K32" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L32" s="2" t="s">
+      <c r="H32" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I32" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="J32" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="N32" s="2" t="s">
-        <v>76</v>
-      </c>
+      <c r="K32" s="2"/>
+      <c r="L32" s="2"/>
+      <c r="M32" s="2"/>
+      <c r="N32" s="2"/>
       <c r="O32" s="2"/>
     </row>
     <row r="33" spans="2:15">
@@ -2171,7 +2175,7 @@
       <c r="G33" s="2"/>
       <c r="H33" s="2"/>
       <c r="I33" s="2"/>
-      <c r="J33" s="2"/>
+      <c r="J33" s="3"/>
       <c r="K33" s="2" t="s">
         <v>20</v>
       </c>
@@ -2179,16 +2183,16 @@
         <v>22</v>
       </c>
       <c r="M33" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N33" s="2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="O33" s="2"/>
     </row>
     <row r="34" spans="2:15">
       <c r="B34" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -2205,52 +2209,42 @@
         <v>22</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="O34" s="2"/>
     </row>
-    <row r="35" spans="2:19">
+    <row r="35" spans="2:15">
       <c r="B35" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D35" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E35" s="2" t="s">
         <v>90</v>
       </c>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
       <c r="F35" s="2"/>
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
       <c r="J35" s="2"/>
-      <c r="K35" s="2"/>
-      <c r="L35" s="2"/>
-      <c r="M35" s="2"/>
-      <c r="N35" s="2"/>
+      <c r="K35" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L35" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M35" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="O35" s="2"/>
-      <c r="P35" t="s">
-        <v>91</v>
-      </c>
-      <c r="Q35" t="s">
-        <v>20</v>
-      </c>
-      <c r="R35" t="s">
-        <v>91</v>
-      </c>
-      <c r="S35" t="s">
-        <v>92</v>
-      </c>
     </row>
     <row r="36" spans="2:19">
       <c r="B36" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C36" s="2" t="s">
         <v>20</v>
@@ -2259,7 +2253,7 @@
         <v>21</v>
       </c>
       <c r="E36" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
@@ -2272,34 +2266,33 @@
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
       <c r="P36" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="Q36" t="s">
         <v>20</v>
       </c>
       <c r="R36" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="S36" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="37" spans="1:16">
-      <c r="A37" t="s">
+    <row r="37" spans="2:19">
+      <c r="B37" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B37" s="2" t="s">
-        <v>96</v>
-      </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>97</v>
-      </c>
+      <c r="C37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F37" s="2"/>
+      <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
@@ -2309,15 +2302,24 @@
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" t="s">
-        <v>98</v>
+        <v>93</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>20</v>
+      </c>
+      <c r="R37" t="s">
+        <v>93</v>
+      </c>
+      <c r="S37" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="38" spans="1:16">
       <c r="A38" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" s="2"/>
@@ -2326,7 +2328,7 @@
         <v>20</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
@@ -2337,84 +2339,99 @@
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="39" spans="2:19">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16">
+      <c r="A39" t="s">
+        <v>97</v>
+      </c>
       <c r="B39" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="H39" s="2"/>
+      <c r="I39" s="2"/>
+      <c r="J39" s="2"/>
+      <c r="K39" s="2"/>
+      <c r="L39" s="2"/>
+      <c r="M39" s="2"/>
+      <c r="N39" s="2"/>
+      <c r="O39" s="2"/>
+      <c r="P39" t="s">
         <v>100</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="D39" s="2" t="s">
+    </row>
+    <row r="40" spans="2:19">
+      <c r="B40" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E39" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="G39" s="2" t="s">
+      <c r="C40" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="H39" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="I39" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="J39" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="K39" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="L39" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="M39" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="N39" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="O39" s="2">
+      <c r="D40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="F40" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="O40" s="2">
         <v>0</v>
       </c>
-      <c r="P39">
+      <c r="P40">
         <v>0</v>
       </c>
-      <c r="Q39" t="s">
-        <v>101</v>
-      </c>
-      <c r="R39">
+      <c r="Q40" t="s">
+        <v>103</v>
+      </c>
+      <c r="R40">
         <v>0</v>
       </c>
-      <c r="S39">
+      <c r="S40">
         <v>0</v>
       </c>
-    </row>
-    <row r="46" spans="1:19">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="N46" s="2"/>
-      <c r="P46" s="2"/>
-      <c r="Q46" s="2"/>
-      <c r="R46" s="2"/>
-      <c r="S46" s="2"/>
     </row>
     <row r="47" spans="1:19">
       <c r="A47" s="2"/>
       <c r="B47" s="2"/>
       <c r="C47" s="2"/>
       <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
       <c r="N47" s="2"/>
-      <c r="O47" s="2"/>
       <c r="P47" s="2"/>
       <c r="Q47" s="2"/>
       <c r="R47" s="2"/>
@@ -2425,6 +2442,7 @@
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
       <c r="N48" s="2"/>
       <c r="O48" s="2"/>
       <c r="P48" s="2"/>
@@ -2564,6 +2582,18 @@
       <c r="R59" s="2"/>
       <c r="S59" s="2"/>
     </row>
+    <row r="60" spans="1:19">
+      <c r="A60" s="2"/>
+      <c r="B60" s="2"/>
+      <c r="C60" s="2"/>
+      <c r="D60" s="2"/>
+      <c r="N60" s="2"/>
+      <c r="O60" s="2"/>
+      <c r="P60" s="2"/>
+      <c r="Q60" s="2"/>
+      <c r="R60" s="2"/>
+      <c r="S60" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  16:24:00 up  7:14,  2 users,  load average: 3.03, 2.78, 2.88
</commit_message>
<xml_diff>
--- a/npc/tools/exu_gen/exu_table.xlsx
+++ b/npc/tools/exu_gen/exu_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="107">
   <si>
     <t>commont</t>
   </si>
@@ -275,6 +275,9 @@
   </si>
   <si>
     <t>8'b00001111</t>
+  </si>
+  <si>
+    <t>`Inst_lb</t>
   </si>
   <si>
     <t>`Inst_sb</t>
@@ -339,9 +342,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
@@ -359,18 +362,11 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF3F3F3F"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -378,14 +374,6 @@
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -397,23 +385,15 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <sz val="18"/>
+      <color theme="3"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -436,7 +416,15 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -448,29 +436,6 @@
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -490,14 +455,52 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF3F3F76"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -524,187 +527,187 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -718,11 +721,32 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -732,15 +756,6 @@
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -762,41 +777,29 @@
     <border>
       <left/>
       <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
       <bottom style="double">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -820,148 +823,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="34" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1312,7 +1315,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S60"/>
+  <dimension ref="A1:S61"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="32.625" customWidth="1"/>
@@ -2168,31 +2171,35 @@
       <c r="B33" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
+      <c r="C33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E33" s="6" t="s">
+        <v>85</v>
+      </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="3"/>
-      <c r="K33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L33" s="2" t="s">
+      <c r="H33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M33" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="N33" s="2" t="s">
+      <c r="J33" s="7" t="s">
         <v>78</v>
       </c>
+      <c r="K33" s="2"/>
+      <c r="L33" s="2"/>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
       <c r="O33" s="2"/>
     </row>
     <row r="34" spans="2:15">
       <c r="B34" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -2201,7 +2208,7 @@
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
+      <c r="J34" s="3"/>
       <c r="K34" s="2" t="s">
         <v>20</v>
       </c>
@@ -2209,10 +2216,10 @@
         <v>22</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="O34" s="2"/>
     </row>
@@ -2235,52 +2242,42 @@
         <v>22</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="O35" s="2"/>
     </row>
-    <row r="36" spans="2:19">
+    <row r="36" spans="2:15">
       <c r="B36" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>92</v>
-      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
-      <c r="N36" s="2"/>
+      <c r="K36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="O36" s="2"/>
-      <c r="P36" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q36" t="s">
-        <v>20</v>
-      </c>
-      <c r="R36" t="s">
-        <v>93</v>
-      </c>
-      <c r="S36" t="s">
-        <v>94</v>
-      </c>
     </row>
     <row r="37" spans="2:19">
       <c r="B37" s="2" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>20</v>
@@ -2289,7 +2286,7 @@
         <v>21</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
@@ -2302,34 +2299,33 @@
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" t="s">
+        <v>94</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>20</v>
+      </c>
+      <c r="R37" t="s">
+        <v>94</v>
+      </c>
+      <c r="S37" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="38" spans="2:19">
+      <c r="B38" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E38" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="Q37" t="s">
-        <v>20</v>
-      </c>
-      <c r="R37" t="s">
-        <v>93</v>
-      </c>
-      <c r="S37" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16">
-      <c r="A38" t="s">
-        <v>97</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>99</v>
-      </c>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
@@ -2339,15 +2335,24 @@
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" t="s">
-        <v>100</v>
+        <v>94</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>20</v>
+      </c>
+      <c r="R38" t="s">
+        <v>94</v>
+      </c>
+      <c r="S38" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="39" spans="1:16">
       <c r="A39" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -2356,7 +2361,7 @@
         <v>20</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
@@ -2367,84 +2372,99 @@
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="40" spans="2:19">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16">
+      <c r="A40" t="s">
+        <v>98</v>
+      </c>
       <c r="B40" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
+      <c r="L40" s="2"/>
+      <c r="M40" s="2"/>
+      <c r="N40" s="2"/>
+      <c r="O40" s="2"/>
+      <c r="P40" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="41" spans="2:19">
+      <c r="B41" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="D40" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E40" s="2" t="s">
+      <c r="D41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="F40" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G40" s="2" t="s">
+      <c r="G41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="I41" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H40" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="I40" s="2" t="s">
+      <c r="J41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="K41" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="J40" s="2" t="s">
+      <c r="L41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="O41" s="2">
+        <v>0</v>
+      </c>
+      <c r="P41">
+        <v>0</v>
+      </c>
+      <c r="Q41" t="s">
         <v>104</v>
       </c>
-      <c r="K40" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="N40" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="O40" s="2">
+      <c r="R41">
         <v>0</v>
       </c>
-      <c r="P40">
+      <c r="S41">
         <v>0</v>
       </c>
-      <c r="Q40" t="s">
-        <v>103</v>
-      </c>
-      <c r="R40">
-        <v>0</v>
-      </c>
-      <c r="S40">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:19">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="N47" s="2"/>
-      <c r="P47" s="2"/>
-      <c r="Q47" s="2"/>
-      <c r="R47" s="2"/>
-      <c r="S47" s="2"/>
     </row>
     <row r="48" spans="1:19">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
       <c r="N48" s="2"/>
-      <c r="O48" s="2"/>
       <c r="P48" s="2"/>
       <c r="Q48" s="2"/>
       <c r="R48" s="2"/>
@@ -2455,6 +2475,7 @@
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
@@ -2594,6 +2615,18 @@
       <c r="R60" s="2"/>
       <c r="S60" s="2"/>
     </row>
+    <row r="61" spans="1:19">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="N61" s="2"/>
+      <c r="O61" s="2"/>
+      <c r="P61" s="2"/>
+      <c r="Q61" s="2"/>
+      <c r="R61" s="2"/>
+      <c r="S61" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  17:21:22 up  8:12,  2 users,  load average: 2.14, 1.52, 1.63
</commit_message>
<xml_diff>
--- a/npc/tools/exu_gen/exu_table.xlsx
+++ b/npc/tools/exu_gen/exu_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="108">
   <si>
     <t>commont</t>
   </si>
@@ -323,6 +323,9 @@
   </si>
   <si>
     <t>`Inst_mret</t>
+  </si>
+  <si>
+    <t>`MEPC_NO</t>
   </si>
   <si>
     <t>default</t>
@@ -1318,7 +1321,7 @@
   <dimension ref="A1:S61"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="32.625" customWidth="1"/>
+    <col min="1" max="1" width="48.9166666666667" customWidth="1"/>
     <col min="2" max="2" width="17.7583333333333" customWidth="1"/>
     <col min="3" max="3" width="10.1416666666667" customWidth="1"/>
     <col min="4" max="4" width="13.1416666666667" customWidth="1"/>
@@ -2400,48 +2403,48 @@
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="41" spans="2:19">
       <c r="B41" s="2" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F41" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E41" s="2" t="s">
+      <c r="G41" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H41" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="F41" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="G41" s="2" t="s">
+      <c r="I41" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="H41" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="I41" s="2" t="s">
+      <c r="J41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K41" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="J41" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>104</v>
-      </c>
       <c r="L41" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="M41" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="N41" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="O41" s="2">
         <v>0</v>
@@ -2450,7 +2453,7 @@
         <v>0</v>
       </c>
       <c r="Q41" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="R41">
         <v>0</v>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  18:41:38 up  9:32,  2 users,  load average: 3.18, 2.60, 2.34
</commit_message>
<xml_diff>
--- a/npc/tools/exu_gen/exu_table.xlsx
+++ b/npc/tools/exu_gen/exu_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="110">
   <si>
     <t>commont</t>
   </si>
@@ -155,6 +155,12 @@
   </si>
   <si>
     <t>$signed(src1) &gt;= $signed(src2) ? imm : 4</t>
+  </si>
+  <si>
+    <t>`Inst_ori</t>
+  </si>
+  <si>
+    <t>src1 | imm</t>
   </si>
   <si>
     <t>`Inst_or</t>
@@ -1318,7 +1324,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S61"/>
+  <dimension ref="A1:S62"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="48.9166666666667" customWidth="1"/>
@@ -1936,7 +1942,7 @@
       <c r="D24" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="2" t="s">
         <v>66</v>
       </c>
       <c r="F24" s="2"/>
@@ -1948,22 +1954,20 @@
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
-      <c r="O24" s="2" t="s">
-        <v>67</v>
-      </c>
+      <c r="O24" s="2"/>
     </row>
     <row r="25" spans="2:15">
       <c r="B25" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1989,7 +1993,7 @@
         <v>21</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -2000,7 +2004,9 @@
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
+      <c r="O26" s="2" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="27" spans="2:15">
       <c r="B27" s="2" t="s">
@@ -2012,7 +2018,7 @@
       <c r="D27" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="4" t="s">
         <v>73</v>
       </c>
       <c r="F27" s="2"/>
@@ -2065,15 +2071,9 @@
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
-      <c r="H29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J29" s="7" t="s">
-        <v>78</v>
-      </c>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
@@ -2082,16 +2082,16 @@
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -2102,7 +2102,7 @@
         <v>22</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
@@ -2112,16 +2112,16 @@
     </row>
     <row r="31" spans="2:15">
       <c r="B31" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E31" s="5" t="s">
-        <v>83</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -2132,7 +2132,7 @@
         <v>22</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
@@ -2150,7 +2150,7 @@
       <c r="D32" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="5" t="s">
         <v>85</v>
       </c>
       <c r="F32" s="2"/>
@@ -2162,7 +2162,7 @@
         <v>22</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
@@ -2172,16 +2172,16 @@
     </row>
     <row r="33" spans="2:15">
       <c r="B33" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E33" s="6" t="s">
         <v>87</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>85</v>
       </c>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
@@ -2192,7 +2192,7 @@
         <v>22</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
@@ -2202,28 +2202,32 @@
     </row>
     <row r="34" spans="2:15">
       <c r="B34" s="2" t="s">
-        <v>88</v>
-      </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
+        <v>89</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E34" s="6" t="s">
+        <v>87</v>
+      </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="3"/>
-      <c r="K34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L34" s="2" t="s">
+      <c r="H34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I34" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M34" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="N34" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="J34" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
       <c r="O34" s="2"/>
     </row>
     <row r="35" spans="2:15">
@@ -2237,7 +2241,7 @@
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
+      <c r="J35" s="3"/>
       <c r="K35" s="2" t="s">
         <v>20</v>
       </c>
@@ -2245,16 +2249,16 @@
         <v>22</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O35" s="2"/>
     </row>
     <row r="36" spans="2:15">
       <c r="B36" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -2271,52 +2275,42 @@
         <v>22</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="O36" s="2"/>
     </row>
-    <row r="37" spans="2:19">
+    <row r="37" spans="2:15">
       <c r="B37" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E37" s="2" t="s">
         <v>93</v>
       </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="2"/>
+      <c r="K37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="O37" s="2"/>
-      <c r="P37" t="s">
-        <v>94</v>
-      </c>
-      <c r="Q37" t="s">
-        <v>20</v>
-      </c>
-      <c r="R37" t="s">
-        <v>94</v>
-      </c>
-      <c r="S37" t="s">
-        <v>95</v>
-      </c>
     </row>
     <row r="38" spans="2:19">
       <c r="B38" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>20</v>
@@ -2325,7 +2319,7 @@
         <v>21</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -2338,34 +2332,33 @@
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="Q38" t="s">
         <v>20</v>
       </c>
       <c r="R38" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="S38" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="39" spans="1:16">
-      <c r="A39" t="s">
+    <row r="39" spans="2:19">
+      <c r="B39" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>100</v>
-      </c>
+      <c r="C39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
@@ -2375,15 +2368,24 @@
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s">
-        <v>101</v>
+        <v>96</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>20</v>
+      </c>
+      <c r="R39" t="s">
+        <v>96</v>
+      </c>
+      <c r="S39" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="40" spans="1:16">
       <c r="A40" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -2392,7 +2394,7 @@
         <v>20</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
@@ -2406,81 +2408,96 @@
         <v>103</v>
       </c>
     </row>
-    <row r="41" spans="2:19">
+    <row r="41" spans="1:16">
+      <c r="A41" t="s">
+        <v>100</v>
+      </c>
       <c r="B41" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C41" s="2" t="s">
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+      <c r="L41" s="2"/>
+      <c r="M41" s="2"/>
+      <c r="N41" s="2"/>
+      <c r="O41" s="2"/>
+      <c r="P41" t="s">
         <v>105</v>
       </c>
-      <c r="D41" s="2" t="s">
+    </row>
+    <row r="42" spans="2:19">
+      <c r="B42" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="G41" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="H41" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="O41" s="2">
+      <c r="D42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="O42" s="2">
         <v>0</v>
       </c>
-      <c r="P41">
+      <c r="P42">
         <v>0</v>
       </c>
-      <c r="Q41" t="s">
-        <v>105</v>
-      </c>
-      <c r="R41">
+      <c r="Q42" t="s">
+        <v>107</v>
+      </c>
+      <c r="R42">
         <v>0</v>
       </c>
-      <c r="S41">
+      <c r="S42">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:19">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="N48" s="2"/>
-      <c r="P48" s="2"/>
-      <c r="Q48" s="2"/>
-      <c r="R48" s="2"/>
-      <c r="S48" s="2"/>
     </row>
     <row r="49" spans="1:19">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
       <c r="N49" s="2"/>
-      <c r="O49" s="2"/>
       <c r="P49" s="2"/>
       <c r="Q49" s="2"/>
       <c r="R49" s="2"/>
@@ -2491,6 +2508,7 @@
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
@@ -2630,6 +2648,18 @@
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
     </row>
+    <row r="62" spans="1:19">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="N62" s="2"/>
+      <c r="O62" s="2"/>
+      <c r="P62" s="2"/>
+      <c r="Q62" s="2"/>
+      <c r="R62" s="2"/>
+      <c r="S62" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
> compile NEMU ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  14:47:41 up  5:05,  2 users,  load average: 0.53, 1.14, 1.33
</commit_message>
<xml_diff>
--- a/npc/tools/exu_gen/exu_table.xlsx
+++ b/npc/tools/exu_gen/exu_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="106">
   <si>
     <t>commont</t>
   </si>
@@ -157,12 +157,6 @@
     <t>$signed(src1) &gt;= $signed(src2) ? imm : 4</t>
   </si>
   <si>
-    <t>`Inst_ori</t>
-  </si>
-  <si>
-    <t>src1 | imm</t>
-  </si>
-  <si>
     <t>`Inst_or</t>
   </si>
   <si>
@@ -283,9 +277,6 @@
     <t>8'b00001111</t>
   </si>
   <si>
-    <t>`Inst_lb</t>
-  </si>
-  <si>
     <t>`Inst_sb</t>
   </si>
   <si>
@@ -329,9 +320,6 @@
   </si>
   <si>
     <t>`Inst_mret</t>
-  </si>
-  <si>
-    <t>`MEPC_NO</t>
   </si>
   <si>
     <t>default</t>
@@ -351,9 +339,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
@@ -371,11 +359,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -383,6 +378,14 @@
       <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -394,15 +397,23 @@
     </font>
     <font>
       <b/>
-      <sz val="18"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="宋体"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FFFF0000"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -425,15 +436,7 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
+      <sz val="18"/>
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -445,6 +448,29 @@
       <color theme="3"/>
       <name val="宋体"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="宋体"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -464,52 +490,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C6500"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF3F3F76"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -536,25 +524,97 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFF2F2F2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -566,7 +626,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -578,43 +668,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -626,97 +704,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -730,32 +718,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -765,6 +732,15 @@
       <top/>
       <bottom style="medium">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -786,29 +762,41 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color theme="4"/>
       </top>
       <bottom style="double">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -832,148 +820,148 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="33" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="18" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="34" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1324,10 +1312,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S62"/>
+  <dimension ref="A1:S60"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
-    <col min="1" max="1" width="48.9166666666667" customWidth="1"/>
+    <col min="1" max="1" width="32.625" customWidth="1"/>
     <col min="2" max="2" width="17.7583333333333" customWidth="1"/>
     <col min="3" max="3" width="10.1416666666667" customWidth="1"/>
     <col min="4" max="4" width="13.1416666666667" customWidth="1"/>
@@ -1942,7 +1930,7 @@
       <c r="D24" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="4" t="s">
         <v>66</v>
       </c>
       <c r="F24" s="2"/>
@@ -1954,11 +1942,13 @@
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
+      <c r="O24" s="2" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="25" spans="2:15">
       <c r="B25" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C25" s="2" t="s">
         <v>20</v>
@@ -1967,7 +1957,7 @@
         <v>21</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1993,7 +1983,7 @@
         <v>21</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -2004,9 +1994,7 @@
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
-      <c r="O26" s="2" t="s">
-        <v>71</v>
-      </c>
+      <c r="O26" s="2"/>
     </row>
     <row r="27" spans="2:15">
       <c r="B27" s="2" t="s">
@@ -2018,7 +2006,7 @@
       <c r="D27" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="4" t="s">
+      <c r="E27" s="2" t="s">
         <v>73</v>
       </c>
       <c r="F27" s="2"/>
@@ -2071,9 +2059,15 @@
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
-      <c r="H29" s="2"/>
-      <c r="I29" s="2"/>
-      <c r="J29" s="2"/>
+      <c r="H29" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="J29" s="7" t="s">
+        <v>78</v>
+      </c>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
@@ -2082,7 +2076,7 @@
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C30" s="2" t="s">
         <v>20</v>
@@ -2091,7 +2085,7 @@
         <v>21</v>
       </c>
       <c r="E30" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -2102,7 +2096,7 @@
         <v>22</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
@@ -2112,7 +2106,7 @@
     </row>
     <row r="31" spans="2:15">
       <c r="B31" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C31" s="2" t="s">
         <v>20</v>
@@ -2120,8 +2114,8 @@
       <c r="D31" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="2" t="s">
-        <v>82</v>
+      <c r="E31" s="5" t="s">
+        <v>83</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -2132,7 +2126,7 @@
         <v>22</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
@@ -2150,7 +2144,7 @@
       <c r="D32" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="E32" s="6" t="s">
         <v>85</v>
       </c>
       <c r="F32" s="2"/>
@@ -2162,7 +2156,7 @@
         <v>22</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
@@ -2172,62 +2166,54 @@
     </row>
     <row r="33" spans="2:15">
       <c r="B33" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E33" s="6" t="s">
         <v>87</v>
       </c>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
-      <c r="H33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I33" s="2" t="s">
+      <c r="H33" s="2"/>
+      <c r="I33" s="2"/>
+      <c r="J33" s="3"/>
+      <c r="K33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J33" s="7" t="s">
+      <c r="M33" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="K33" s="2"/>
-      <c r="L33" s="2"/>
-      <c r="M33" s="2"/>
-      <c r="N33" s="2"/>
+      <c r="N33" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="O33" s="2"/>
     </row>
     <row r="34" spans="2:15">
       <c r="B34" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D34" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>87</v>
-      </c>
+      <c r="C34" s="2"/>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
-      <c r="H34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I34" s="2" t="s">
+      <c r="H34" s="2"/>
+      <c r="I34" s="2"/>
+      <c r="J34" s="2"/>
+      <c r="K34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L34" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="J34" s="7" t="s">
-        <v>80</v>
-      </c>
-      <c r="K34" s="2"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="2"/>
-      <c r="N34" s="2"/>
+      <c r="M34" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="O34" s="2"/>
     </row>
     <row r="35" spans="2:15">
@@ -2241,7 +2227,7 @@
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
-      <c r="J35" s="3"/>
+      <c r="J35" s="2"/>
       <c r="K35" s="2" t="s">
         <v>20</v>
       </c>
@@ -2249,80 +2235,101 @@
         <v>22</v>
       </c>
       <c r="M35" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="O35" s="2"/>
+    </row>
+    <row r="36" spans="2:19">
+      <c r="B36" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="N35" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="O35" s="2"/>
-    </row>
-    <row r="36" spans="2:15">
-      <c r="B36" s="2" t="s">
+      <c r="C36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="K36" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L36" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M36" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="N36" s="2" t="s">
-        <v>83</v>
-      </c>
+      <c r="K36" s="2"/>
+      <c r="L36" s="2"/>
+      <c r="M36" s="2"/>
+      <c r="N36" s="2"/>
       <c r="O36" s="2"/>
-    </row>
-    <row r="37" spans="2:15">
+      <c r="P36" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>20</v>
+      </c>
+      <c r="R36" t="s">
+        <v>93</v>
+      </c>
+      <c r="S36" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="37" spans="2:19">
       <c r="B37" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
+        <v>95</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E37" s="2" t="s">
+        <v>92</v>
+      </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
-      <c r="K37" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L37" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="M37" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="N37" s="2" t="s">
-        <v>88</v>
-      </c>
+      <c r="K37" s="2"/>
+      <c r="L37" s="2"/>
+      <c r="M37" s="2"/>
+      <c r="N37" s="2"/>
       <c r="O37" s="2"/>
-    </row>
-    <row r="38" spans="2:19">
+      <c r="P37" t="s">
+        <v>93</v>
+      </c>
+      <c r="Q37" t="s">
+        <v>20</v>
+      </c>
+      <c r="R37" t="s">
+        <v>93</v>
+      </c>
+      <c r="S37" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="38" spans="1:16">
+      <c r="A38" t="s">
+        <v>97</v>
+      </c>
       <c r="B38" s="2" t="s">
-        <v>94</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E38" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F38" s="2"/>
-      <c r="G38" s="2"/>
+        <v>98</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>99</v>
+      </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
@@ -2332,33 +2339,25 @@
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q38" t="s">
-        <v>20</v>
-      </c>
-      <c r="R38" t="s">
-        <v>96</v>
-      </c>
-      <c r="S38" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="39" spans="1:16">
+      <c r="A39" t="s">
         <v>97</v>
       </c>
-    </row>
-    <row r="39" spans="2:19">
       <c r="B39" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="F39" s="2"/>
-      <c r="G39" s="2"/>
+        <v>101</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>99</v>
+      </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
@@ -2368,129 +2367,88 @@
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s">
-        <v>96</v>
-      </c>
-      <c r="Q39" t="s">
-        <v>20</v>
-      </c>
-      <c r="R39" t="s">
-        <v>96</v>
-      </c>
-      <c r="S39" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16">
-      <c r="A40" t="s">
         <v>100</v>
       </c>
+    </row>
+    <row r="40" spans="2:19">
       <c r="B40" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
+        <v>102</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E40" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="F40" s="2" t="s">
-        <v>20</v>
+        <v>103</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="H40" s="2"/>
-      <c r="I40" s="2"/>
-      <c r="J40" s="2"/>
-      <c r="K40" s="2"/>
-      <c r="L40" s="2"/>
-      <c r="M40" s="2"/>
-      <c r="N40" s="2"/>
-      <c r="O40" s="2"/>
-      <c r="P40" t="s">
+        <v>105</v>
+      </c>
+      <c r="H40" s="2" t="s">
         <v>103</v>
       </c>
-    </row>
-    <row r="41" spans="1:16">
-      <c r="A41" t="s">
-        <v>100</v>
-      </c>
-      <c r="B41" s="2" t="s">
+      <c r="I40" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G41" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="H41" s="2"/>
-      <c r="I41" s="2"/>
-      <c r="J41" s="2"/>
-      <c r="K41" s="2"/>
-      <c r="L41" s="2"/>
-      <c r="M41" s="2"/>
-      <c r="N41" s="2"/>
-      <c r="O41" s="2"/>
-      <c r="P41" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="42" spans="2:19">
-      <c r="B42" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="D42" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="E42" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="F42" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G42" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="I42" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="J42" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="L42" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="M42" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="N42" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="O42" s="2">
+      <c r="J40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="K40" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="L40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="M40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="O40" s="2">
         <v>0</v>
       </c>
-      <c r="P42">
+      <c r="P40">
         <v>0</v>
       </c>
-      <c r="Q42" t="s">
-        <v>107</v>
-      </c>
-      <c r="R42">
+      <c r="Q40" t="s">
+        <v>103</v>
+      </c>
+      <c r="R40">
         <v>0</v>
       </c>
-      <c r="S42">
+      <c r="S40">
         <v>0</v>
       </c>
+    </row>
+    <row r="47" spans="1:19">
+      <c r="A47" s="2"/>
+      <c r="B47" s="2"/>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="N47" s="2"/>
+      <c r="P47" s="2"/>
+      <c r="Q47" s="2"/>
+      <c r="R47" s="2"/>
+      <c r="S47" s="2"/>
+    </row>
+    <row r="48" spans="1:19">
+      <c r="A48" s="2"/>
+      <c r="B48" s="2"/>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="N48" s="2"/>
+      <c r="O48" s="2"/>
+      <c r="P48" s="2"/>
+      <c r="Q48" s="2"/>
+      <c r="R48" s="2"/>
+      <c r="S48" s="2"/>
     </row>
     <row r="49" spans="1:19">
       <c r="A49" s="2"/>
@@ -2498,6 +2456,7 @@
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
       <c r="N49" s="2"/>
+      <c r="O49" s="2"/>
       <c r="P49" s="2"/>
       <c r="Q49" s="2"/>
       <c r="R49" s="2"/>
@@ -2508,7 +2467,6 @@
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
@@ -2636,30 +2594,6 @@
       <c r="R60" s="2"/>
       <c r="S60" s="2"/>
     </row>
-    <row r="61" spans="1:19">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="N61" s="2"/>
-      <c r="O61" s="2"/>
-      <c r="P61" s="2"/>
-      <c r="Q61" s="2"/>
-      <c r="R61" s="2"/>
-      <c r="S61" s="2"/>
-    </row>
-    <row r="62" spans="1:19">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="N62" s="2"/>
-      <c r="O62" s="2"/>
-      <c r="P62" s="2"/>
-      <c r="Q62" s="2"/>
-      <c r="R62" s="2"/>
-      <c r="S62" s="2"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  15:00:42 up  5:18,  2 users,  load average: 1.32, 1.93, 1.81
</commit_message>
<xml_diff>
--- a/npc/tools/exu_gen/exu_table.xlsx
+++ b/npc/tools/exu_gen/exu_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="108">
   <si>
     <t>commont</t>
   </si>
@@ -260,6 +260,12 @@
   </si>
   <si>
     <t>8'b00000011</t>
+  </si>
+  <si>
+    <t>`Inst_lb</t>
+  </si>
+  <si>
+    <t>{{(`WordWidth-8){mem_r_data[7]}}, mem_r_data[7:0]}</t>
   </si>
   <si>
     <t>`Inst_lh</t>
@@ -359,8 +365,30 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <u/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF0000FF"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -375,37 +403,22 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF006100"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <i/>
       <sz val="11"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF7F7F7F"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF9C0006"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -419,30 +432,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="宋体"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="15"/>
       <color theme="3"/>
@@ -453,37 +442,15 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="3"/>
       <name val="宋体"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="宋体"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
       <name val="宋体"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -502,6 +469,45 @@
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="宋体"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="宋体"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="35">
     <fill>
@@ -524,36 +530,174 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -566,145 +710,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -715,15 +721,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -738,9 +735,35 @@
     <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -760,13 +783,26 @@
       <diagonal/>
     </border>
     <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
+      <top/>
       <bottom style="double">
-        <color theme="4"/>
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -785,183 +821,153 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="25" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="33" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="4" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="28" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="28" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="34" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1312,7 +1318,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S60"/>
+  <dimension ref="A1:S61"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="32.625" customWidth="1"/>
@@ -2114,7 +2120,7 @@
       <c r="D31" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E31" s="5" t="s">
+      <c r="E31" s="2" t="s">
         <v>83</v>
       </c>
       <c r="F31" s="2"/>
@@ -2126,7 +2132,7 @@
         <v>22</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
@@ -2144,7 +2150,7 @@
       <c r="D32" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="6" t="s">
+      <c r="E32" s="5" t="s">
         <v>85</v>
       </c>
       <c r="F32" s="2"/>
@@ -2156,7 +2162,7 @@
         <v>22</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
@@ -2166,28 +2172,32 @@
     </row>
     <row r="33" spans="2:15">
       <c r="B33" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D33" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E33" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
-      <c r="H33" s="2"/>
-      <c r="I33" s="2"/>
-      <c r="J33" s="3"/>
-      <c r="K33" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L33" s="2" t="s">
+      <c r="H33" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M33" s="2" t="s">
+      <c r="J33" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="N33" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="K33" s="2"/>
+      <c r="L33" s="2"/>
+      <c r="M33" s="2"/>
+      <c r="N33" s="2"/>
       <c r="O33" s="2"/>
     </row>
     <row r="34" spans="2:15">
@@ -2201,7 +2211,7 @@
       <c r="G34" s="2"/>
       <c r="H34" s="2"/>
       <c r="I34" s="2"/>
-      <c r="J34" s="2"/>
+      <c r="J34" s="3"/>
       <c r="K34" s="2" t="s">
         <v>20</v>
       </c>
@@ -2209,16 +2219,16 @@
         <v>22</v>
       </c>
       <c r="M34" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="N34" s="2" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="O34" s="2"/>
     </row>
     <row r="35" spans="2:15">
       <c r="B35" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -2235,52 +2245,42 @@
         <v>22</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="O35" s="2"/>
     </row>
-    <row r="36" spans="2:19">
+    <row r="36" spans="2:15">
       <c r="B36" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E36" s="2" t="s">
         <v>92</v>
       </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
       <c r="F36" s="2"/>
       <c r="G36" s="2"/>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
       <c r="J36" s="2"/>
-      <c r="K36" s="2"/>
-      <c r="L36" s="2"/>
-      <c r="M36" s="2"/>
-      <c r="N36" s="2"/>
+      <c r="K36" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L36" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M36" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>88</v>
+      </c>
       <c r="O36" s="2"/>
-      <c r="P36" t="s">
-        <v>93</v>
-      </c>
-      <c r="Q36" t="s">
-        <v>20</v>
-      </c>
-      <c r="R36" t="s">
-        <v>93</v>
-      </c>
-      <c r="S36" t="s">
-        <v>94</v>
-      </c>
     </row>
     <row r="37" spans="2:19">
       <c r="B37" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C37" s="2" t="s">
         <v>20</v>
@@ -2289,7 +2289,7 @@
         <v>21</v>
       </c>
       <c r="E37" s="2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
@@ -2302,34 +2302,33 @@
       <c r="N37" s="2"/>
       <c r="O37" s="2"/>
       <c r="P37" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="Q37" t="s">
         <v>20</v>
       </c>
       <c r="R37" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="S37" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="38" spans="1:16">
-      <c r="A38" t="s">
+    <row r="38" spans="2:19">
+      <c r="B38" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B38" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>99</v>
-      </c>
+      <c r="C38" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="F38" s="2"/>
+      <c r="G38" s="2"/>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
       <c r="J38" s="2"/>
@@ -2339,15 +2338,24 @@
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" t="s">
-        <v>100</v>
+        <v>95</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>20</v>
+      </c>
+      <c r="R38" t="s">
+        <v>95</v>
+      </c>
+      <c r="S38" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:16">
       <c r="A39" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
@@ -2356,7 +2364,7 @@
         <v>20</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
@@ -2367,84 +2375,99 @@
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="40" spans="2:19">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="40" spans="1:16">
+      <c r="A40" t="s">
+        <v>99</v>
+      </c>
       <c r="B40" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H40" s="2"/>
+      <c r="I40" s="2"/>
+      <c r="J40" s="2"/>
+      <c r="K40" s="2"/>
+      <c r="L40" s="2"/>
+      <c r="M40" s="2"/>
+      <c r="N40" s="2"/>
+      <c r="O40" s="2"/>
+      <c r="P40" t="s">
         <v>102</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D40" s="2" t="s">
+    </row>
+    <row r="41" spans="2:19">
+      <c r="B41" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="E40" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G40" s="2" t="s">
+      <c r="C41" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="H40" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="I40" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="J40" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="K40" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="M40" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="N40" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="O40" s="2">
+      <c r="D41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="F41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="I41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="K41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="L41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="M41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>106</v>
+      </c>
+      <c r="O41" s="2">
         <v>0</v>
       </c>
-      <c r="P40">
+      <c r="P41">
         <v>0</v>
       </c>
-      <c r="Q40" t="s">
-        <v>103</v>
-      </c>
-      <c r="R40">
+      <c r="Q41" t="s">
+        <v>105</v>
+      </c>
+      <c r="R41">
         <v>0</v>
       </c>
-      <c r="S40">
+      <c r="S41">
         <v>0</v>
       </c>
-    </row>
-    <row r="47" spans="1:19">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="N47" s="2"/>
-      <c r="P47" s="2"/>
-      <c r="Q47" s="2"/>
-      <c r="R47" s="2"/>
-      <c r="S47" s="2"/>
     </row>
     <row r="48" spans="1:19">
       <c r="A48" s="2"/>
       <c r="B48" s="2"/>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
       <c r="N48" s="2"/>
-      <c r="O48" s="2"/>
       <c r="P48" s="2"/>
       <c r="Q48" s="2"/>
       <c r="R48" s="2"/>
@@ -2455,6 +2478,7 @@
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
       <c r="N49" s="2"/>
       <c r="O49" s="2"/>
       <c r="P49" s="2"/>
@@ -2594,6 +2618,18 @@
       <c r="R60" s="2"/>
       <c r="S60" s="2"/>
     </row>
+    <row r="61" spans="1:19">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="N61" s="2"/>
+      <c r="O61" s="2"/>
+      <c r="P61" s="2"/>
+      <c r="Q61" s="2"/>
+      <c r="R61" s="2"/>
+      <c r="S61" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  15:10:33 up  5:27,  2 users,  load average: 2.06, 2.23, 1.92
</commit_message>
<xml_diff>
--- a/npc/tools/exu_gen/exu_table.xlsx
+++ b/npc/tools/exu_gen/exu_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="110">
   <si>
     <t>commont</t>
   </si>
@@ -89,6 +89,12 @@
   </si>
   <si>
     <t>src1 &amp; imm</t>
+  </si>
+  <si>
+    <t>`Inst_ori</t>
+  </si>
+  <si>
+    <t>src1 | imm</t>
   </si>
   <si>
     <t>`Inst_xori</t>
@@ -1318,7 +1324,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:S61"/>
+  <dimension ref="A1:S62"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="32.625" customWidth="1"/>
@@ -1520,34 +1526,29 @@
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
     </row>
-    <row r="7" s="1" customFormat="1" spans="1:15">
-      <c r="A7"/>
-      <c r="B7" s="3" t="s">
+    <row r="7" spans="2:15">
+      <c r="B7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="3" t="s">
+      <c r="C7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F7" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
     </row>
     <row r="8" s="1" customFormat="1" spans="1:15">
       <c r="A8"/>
@@ -1561,13 +1562,13 @@
         <v>21</v>
       </c>
       <c r="E8" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G8" s="3" t="s">
         <v>32</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>34</v>
       </c>
       <c r="H8" s="3"/>
       <c r="I8" s="3"/>
@@ -1578,27 +1579,34 @@
       <c r="N8" s="3"/>
       <c r="O8" s="3"/>
     </row>
-    <row r="9" spans="2:15">
-      <c r="B9" s="2" t="s">
+    <row r="9" s="1" customFormat="1" spans="1:15">
+      <c r="A9"/>
+      <c r="B9" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="2" t="s">
+      <c r="C9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G9" s="3" t="s">
         <v>36</v>
       </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
+      <c r="O9" s="3"/>
     </row>
     <row r="10" spans="2:15">
       <c r="B10" s="2" t="s">
@@ -1714,17 +1722,15 @@
       <c r="B15" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D15" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E15" s="2" t="s">
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G15" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -1936,7 +1942,7 @@
       <c r="D24" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E24" s="4" t="s">
+      <c r="E24" s="2" t="s">
         <v>66</v>
       </c>
       <c r="F24" s="2"/>
@@ -1948,22 +1954,20 @@
       <c r="L24" s="2"/>
       <c r="M24" s="2"/>
       <c r="N24" s="2"/>
-      <c r="O24" s="2" t="s">
-        <v>67</v>
-      </c>
+      <c r="O24" s="2"/>
     </row>
     <row r="25" spans="2:15">
       <c r="B25" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E25" s="4" t="s">
         <v>68</v>
-      </c>
-      <c r="C25" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D25" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E25" s="4" t="s">
-        <v>66</v>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>
@@ -1989,7 +1993,7 @@
         <v>21</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2"/>
@@ -2000,7 +2004,9 @@
       <c r="L26" s="2"/>
       <c r="M26" s="2"/>
       <c r="N26" s="2"/>
-      <c r="O26" s="2"/>
+      <c r="O26" s="2" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="27" spans="2:15">
       <c r="B27" s="2" t="s">
@@ -2012,7 +2018,7 @@
       <c r="D27" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="4" t="s">
         <v>73</v>
       </c>
       <c r="F27" s="2"/>
@@ -2065,15 +2071,9 @@
       </c>
       <c r="F29" s="2"/>
       <c r="G29" s="2"/>
-      <c r="H29" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="J29" s="7" t="s">
-        <v>78</v>
-      </c>
+      <c r="H29" s="2"/>
+      <c r="I29" s="2"/>
+      <c r="J29" s="2"/>
       <c r="K29" s="2"/>
       <c r="L29" s="2"/>
       <c r="M29" s="2"/>
@@ -2082,16 +2082,16 @@
     </row>
     <row r="30" spans="2:15">
       <c r="B30" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D30" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>79</v>
-      </c>
-      <c r="C30" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D30" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E30" s="2" t="s">
-        <v>80</v>
       </c>
       <c r="F30" s="2"/>
       <c r="G30" s="2"/>
@@ -2102,7 +2102,7 @@
         <v>22</v>
       </c>
       <c r="J30" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K30" s="2"/>
       <c r="L30" s="2"/>
@@ -2112,16 +2112,16 @@
     </row>
     <row r="31" spans="2:15">
       <c r="B31" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D31" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>82</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>83</v>
       </c>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -2132,7 +2132,7 @@
         <v>22</v>
       </c>
       <c r="J31" s="7" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="K31" s="2"/>
       <c r="L31" s="2"/>
@@ -2150,7 +2150,7 @@
       <c r="D32" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="E32" s="2" t="s">
         <v>85</v>
       </c>
       <c r="F32" s="2"/>
@@ -2162,7 +2162,7 @@
         <v>22</v>
       </c>
       <c r="J32" s="7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="K32" s="2"/>
       <c r="L32" s="2"/>
@@ -2180,7 +2180,7 @@
       <c r="D33" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="E33" s="6" t="s">
+      <c r="E33" s="5" t="s">
         <v>87</v>
       </c>
       <c r="F33" s="2"/>
@@ -2192,7 +2192,7 @@
         <v>22</v>
       </c>
       <c r="J33" s="7" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="K33" s="2"/>
       <c r="L33" s="2"/>
@@ -2202,28 +2202,32 @@
     </row>
     <row r="34" spans="2:15">
       <c r="B34" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E34" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="C34" s="2"/>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
       <c r="F34" s="2"/>
       <c r="G34" s="2"/>
-      <c r="H34" s="2"/>
-      <c r="I34" s="2"/>
-      <c r="J34" s="3"/>
-      <c r="K34" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="L34" s="2" t="s">
+      <c r="H34" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I34" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="M34" s="2" t="s">
+      <c r="J34" s="7" t="s">
         <v>90</v>
       </c>
-      <c r="N34" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="K34" s="2"/>
+      <c r="L34" s="2"/>
+      <c r="M34" s="2"/>
+      <c r="N34" s="2"/>
       <c r="O34" s="2"/>
     </row>
     <row r="35" spans="2:15">
@@ -2237,7 +2241,7 @@
       <c r="G35" s="2"/>
       <c r="H35" s="2"/>
       <c r="I35" s="2"/>
-      <c r="J35" s="2"/>
+      <c r="J35" s="3"/>
       <c r="K35" s="2" t="s">
         <v>20</v>
       </c>
@@ -2245,16 +2249,16 @@
         <v>22</v>
       </c>
       <c r="M35" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="N35" s="2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="O35" s="2"/>
     </row>
     <row r="36" spans="2:15">
       <c r="B36" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -2271,52 +2275,42 @@
         <v>22</v>
       </c>
       <c r="M36" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="N36" s="2" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="O36" s="2"/>
     </row>
-    <row r="37" spans="2:19">
+    <row r="37" spans="2:15">
       <c r="B37" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E37" s="2" t="s">
         <v>94</v>
       </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
       <c r="F37" s="2"/>
       <c r="G37" s="2"/>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
       <c r="J37" s="2"/>
-      <c r="K37" s="2"/>
-      <c r="L37" s="2"/>
-      <c r="M37" s="2"/>
-      <c r="N37" s="2"/>
+      <c r="K37" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="L37" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>90</v>
+      </c>
       <c r="O37" s="2"/>
-      <c r="P37" t="s">
-        <v>95</v>
-      </c>
-      <c r="Q37" t="s">
-        <v>20</v>
-      </c>
-      <c r="R37" t="s">
-        <v>95</v>
-      </c>
-      <c r="S37" t="s">
-        <v>96</v>
-      </c>
     </row>
     <row r="38" spans="2:19">
       <c r="B38" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C38" s="2" t="s">
         <v>20</v>
@@ -2325,7 +2319,7 @@
         <v>21</v>
       </c>
       <c r="E38" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -2338,34 +2332,33 @@
       <c r="N38" s="2"/>
       <c r="O38" s="2"/>
       <c r="P38" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="Q38" t="s">
         <v>20</v>
       </c>
       <c r="R38" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="S38" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="39" spans="1:16">
-      <c r="A39" t="s">
+    <row r="39" spans="2:19">
+      <c r="B39" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B39" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
-      <c r="F39" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>101</v>
-      </c>
+      <c r="C39" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E39" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="F39" s="2"/>
+      <c r="G39" s="2"/>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
@@ -2375,15 +2368,24 @@
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
       <c r="P39" t="s">
-        <v>102</v>
+        <v>97</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>20</v>
+      </c>
+      <c r="R39" t="s">
+        <v>97</v>
+      </c>
+      <c r="S39" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="40" spans="1:16">
       <c r="A40" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -2392,7 +2394,7 @@
         <v>20</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
@@ -2403,84 +2405,99 @@
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
       <c r="P40" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="41" spans="2:19">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="41" spans="1:16">
+      <c r="A41" t="s">
+        <v>101</v>
+      </c>
       <c r="B41" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="H41" s="2"/>
+      <c r="I41" s="2"/>
+      <c r="J41" s="2"/>
+      <c r="K41" s="2"/>
+      <c r="L41" s="2"/>
+      <c r="M41" s="2"/>
+      <c r="N41" s="2"/>
+      <c r="O41" s="2"/>
+      <c r="P41" t="s">
         <v>104</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="D41" s="2" t="s">
+    </row>
+    <row r="42" spans="2:19">
+      <c r="B42" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="F41" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="G41" s="2" t="s">
+      <c r="C42" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="H41" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="I41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="J41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="K41" s="2" t="s">
-        <v>105</v>
-      </c>
-      <c r="L41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="M41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="N41" s="2" t="s">
-        <v>106</v>
-      </c>
-      <c r="O41" s="2">
+      <c r="D42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="F42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="K42" s="2" t="s">
+        <v>107</v>
+      </c>
+      <c r="L42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="M42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="O42" s="2">
         <v>0</v>
       </c>
-      <c r="P41">
+      <c r="P42">
         <v>0</v>
       </c>
-      <c r="Q41" t="s">
-        <v>105</v>
-      </c>
-      <c r="R41">
+      <c r="Q42" t="s">
+        <v>107</v>
+      </c>
+      <c r="R42">
         <v>0</v>
       </c>
-      <c r="S41">
+      <c r="S42">
         <v>0</v>
       </c>
-    </row>
-    <row r="48" spans="1:19">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="N48" s="2"/>
-      <c r="P48" s="2"/>
-      <c r="Q48" s="2"/>
-      <c r="R48" s="2"/>
-      <c r="S48" s="2"/>
     </row>
     <row r="49" spans="1:19">
       <c r="A49" s="2"/>
       <c r="B49" s="2"/>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
       <c r="N49" s="2"/>
-      <c r="O49" s="2"/>
       <c r="P49" s="2"/>
       <c r="Q49" s="2"/>
       <c r="R49" s="2"/>
@@ -2491,6 +2508,7 @@
       <c r="B50" s="2"/>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
       <c r="N50" s="2"/>
       <c r="O50" s="2"/>
       <c r="P50" s="2"/>
@@ -2630,6 +2648,18 @@
       <c r="R61" s="2"/>
       <c r="S61" s="2"/>
     </row>
+    <row r="62" spans="1:19">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="N62" s="2"/>
+      <c r="O62" s="2"/>
+      <c r="P62" s="2"/>
+      <c r="Q62" s="2"/>
+      <c r="R62" s="2"/>
+      <c r="S62" s="2"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
> sim RTL ysyx_23060246 韩炳晋 Linux archlinux 6.6.60-1-lts #1 SMP PREEMPT_DYNAMIC Fri, 08 Nov 2024 16:03:02 +0000 x86_64 GNU/Linux  15:22:09 up  5:39,  2 users,  load average: 0.51, 0.64, 1.11
</commit_message>
<xml_diff>
--- a/npc/tools/exu_gen/exu_table.xlsx
+++ b/npc/tools/exu_gen/exu_table.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="111">
   <si>
     <t>commont</t>
   </si>
@@ -332,6 +332,9 @@
   </si>
   <si>
     <t>`Inst_mret</t>
+  </si>
+  <si>
+    <t>`MEPC_NO</t>
   </si>
   <si>
     <t>default</t>
@@ -2433,48 +2436,48 @@
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
       <c r="P41" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
     </row>
     <row r="42" spans="2:19">
       <c r="B42" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D42" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E42" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="F42" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="E42" s="2" t="s">
+      <c r="G42" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="H42" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="F42" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G42" s="2" t="s">
+      <c r="I42" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="H42" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="I42" s="2" t="s">
+      <c r="J42" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="K42" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="J42" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="K42" s="2" t="s">
-        <v>107</v>
-      </c>
       <c r="L42" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="M42" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="N42" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="O42" s="2">
         <v>0</v>
@@ -2483,7 +2486,7 @@
         <v>0</v>
       </c>
       <c r="Q42" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="R42">
         <v>0</v>

</xml_diff>